<commit_message>
feat(location): auto save user location on login
</commit_message>
<xml_diff>
--- a/ThoDenNgay_Product_Bible.xlsx
+++ b/ThoDenNgay_Product_Bible.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\alo-tho-master\alo-tho-master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF048375-3B95-4446-9DD8-20DF16F7319D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80D0DE4A-675D-4E02-9AC5-796419FADED7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{BA8B2107-ECAC-46C3-9034-2B15E763C8B5}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="36">
   <si>
     <t>STT</t>
   </si>
@@ -94,6 +94,54 @@
   </si>
   <si>
     <t>Separate BillGo module from customer management</t>
+  </si>
+  <si>
+    <t>GPS đăng nhập</t>
+  </si>
+  <si>
+    <t>Khách và thợ tự động cập nhật GPS sau đăng nhập</t>
+  </si>
+  <si>
+    <t>Chỉ ghi khi di chuyển trên 100m hoặc quá 5 phút</t>
+  </si>
+  <si>
+    <t>feat(location): auto save user location on login</t>
+  </si>
+  <si>
+    <t>Khách hàng / Thợ</t>
+  </si>
+  <si>
+    <t>Yêu cầu quyền vị trí sau xác thực; từ chối vẫn vào ứng dụng</t>
+  </si>
+  <si>
+    <t>Không làm gián đoạn đăng nhập</t>
+  </si>
+  <si>
+    <t>profiles location</t>
+  </si>
+  <si>
+    <t>latitude, longitude, last_location_at, location_updated_by</t>
+  </si>
+  <si>
+    <t>Giữ gps_location để tương thích luồng cũ</t>
+  </si>
+  <si>
+    <t>GPS best-effort</t>
+  </si>
+  <si>
+    <t>Không chặn đăng nhập khi thiếu quyền hoặc GPS lỗi</t>
+  </si>
+  <si>
+    <t>Tôn trọng quyền riêng tư và độ ổn định</t>
+  </si>
+  <si>
+    <t>Auto save login location</t>
+  </si>
+  <si>
+    <t>Tập trung logic tại services/locationService.ts</t>
+  </si>
+  <si>
+    <t>Khoảng cách và phân công thợ dùng vị trí mới hơn</t>
   </si>
 </sst>
 </file>
@@ -499,12 +547,12 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2631304A-15A0-4692-B08D-1B98A6A6FAC0}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="53.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="47.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="48.7109375" bestFit="1" customWidth="1"/>
@@ -550,6 +598,26 @@
         <v>19</v>
       </c>
     </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F3" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -557,15 +625,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEC9037B-EFE6-49F5-A5F3-F97E00C66B25}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="78" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="43.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="43.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -602,6 +670,26 @@
         <v>7</v>
       </c>
     </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -609,15 +697,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FE72BEA-FB82-4065-A82E-8E80ACFB3A0B}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="70.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="43.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -654,6 +742,26 @@
         <v>9</v>
       </c>
     </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F3" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -661,15 +769,15 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73AD43CE-C0B8-4E8A-BE78-46E5E8BA5D1B}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="114.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="37.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="43.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -707,6 +815,26 @@
       </c>
       <c r="E2" t="s">
         <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -754,15 +882,15 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A759B5AA-E445-44B2-84E8-3B69A2E43B9A}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="57.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="32.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="43.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -800,6 +928,26 @@
       </c>
       <c r="E2" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F3" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: support multi-service job with hierarchical service selector
</commit_message>
<xml_diff>
--- a/ThoDenNgay_Product_Bible.xlsx
+++ b/ThoDenNgay_Product_Bible.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\alo-tho-master\alo-tho-master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80D0DE4A-675D-4E02-9AC5-796419FADED7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BF80788-47CD-40E3-8FC9-638E162C3E51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{BA8B2107-ECAC-46C3-9034-2B15E763C8B5}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="52">
   <si>
     <t>STT</t>
   </si>
@@ -142,6 +142,54 @@
   </si>
   <si>
     <t>Khoảng cách và phân công thợ dùng vị trí mới hơn</t>
+  </si>
+  <si>
+    <t>Multi-service job</t>
+  </si>
+  <si>
+    <t>Chọn nhiều dịch vụ bằng cây Parent → Child tại khách, thợ và admin</t>
+  </si>
+  <si>
+    <t>Danh mục cha chỉ mở/đóng; dịch vụ lá được chọn</t>
+  </si>
+  <si>
+    <t>feat: support multi-service job with hierarchical service selector</t>
+  </si>
+  <si>
+    <t>Khách hàng / Thợ / Admin</t>
+  </si>
+  <si>
+    <t>Một phiếu việc có nhiều dịch vụ và workflow hợp nhất</t>
+  </si>
+  <si>
+    <t>Dịch vụ trùng chỉ lưu một quan hệ</t>
+  </si>
+  <si>
+    <t>job_services</t>
+  </si>
+  <si>
+    <t>Quan hệ nhiều-nhiều; giữ jobs.service_id làm primary/fallback</t>
+  </si>
+  <si>
+    <t>Không xóa hoặc đổi dữ liệu legacy</t>
+  </si>
+  <si>
+    <t>Hierarchical service selector</t>
+  </si>
+  <si>
+    <t>Dùng component cây checkbox thay dropdown dài</t>
+  </si>
+  <si>
+    <t>Tối ưu mobile và mở rộng danh mục</t>
+  </si>
+  <si>
+    <t>Multi-service hierarchical selector</t>
+  </si>
+  <si>
+    <t>Đồng bộ UI chọn và màn hình đọc chi tiết</t>
+  </si>
+  <si>
+    <t>BillGo/workflow tiếp tục dựa trên primary + danh sách services</t>
   </si>
 </sst>
 </file>
@@ -547,15 +595,15 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2631304A-15A0-4692-B08D-1B98A6A6FAC0}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="53.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="47.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="48.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="57.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="59" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -618,6 +666,26 @@
         <v>23</v>
       </c>
     </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4" t="s">
+        <v>50</v>
+      </c>
+      <c r="E4" t="s">
+        <v>51</v>
+      </c>
+      <c r="F4" t="s">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -625,15 +693,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEC9037B-EFE6-49F5-A5F3-F97E00C66B25}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="78" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="43.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="43.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="44.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="59" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -690,6 +758,26 @@
         <v>23</v>
       </c>
     </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D4" t="s">
+        <v>37</v>
+      </c>
+      <c r="E4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4" t="s">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -697,15 +785,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FE72BEA-FB82-4065-A82E-8E80ACFB3A0B}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="70.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="43.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="59" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -762,6 +850,26 @@
         <v>23</v>
       </c>
     </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E4" t="s">
+        <v>42</v>
+      </c>
+      <c r="F4" t="s">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -769,7 +877,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73AD43CE-C0B8-4E8A-BE78-46E5E8BA5D1B}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -777,7 +885,7 @@
     <col min="3" max="3" width="22.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="114.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="37.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="43.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="59" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -835,6 +943,26 @@
       </c>
       <c r="F3" t="s">
         <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E4" t="s">
+        <v>45</v>
+      </c>
+      <c r="F4" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -882,15 +1010,15 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A759B5AA-E445-44B2-84E8-3B69A2E43B9A}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="57.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="36" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="43.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="59" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -948,6 +1076,26 @@
       </c>
       <c r="F3" t="s">
         <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F4" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(worker): add feature registry and dynamic module menu system
</commit_message>
<xml_diff>
--- a/ThoDenNgay_Product_Bible.xlsx
+++ b/ThoDenNgay_Product_Bible.xlsx
@@ -594,9 +594,9 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2631304A-15A0-4692-B08D-1B98A6A6FAC0}">
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{2631304A-15A0-4692-B08D-1B98A6A6FAC0}">
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
@@ -606,7 +606,7 @@
     <col min="6" max="6" width="59" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" s="1" customFormat="1" ns3:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -626,7 +626,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ns3:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -646,7 +646,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ns3:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -666,7 +666,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ns3:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -684,6 +684,34 @@
       </c>
       <c r="F4" t="s">
         <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Commit 1 Worker Feature Registry</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Da xay dung registry va menu dong cho trang Tho; BillGo an/hien theo du lieu thuc te.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Khong thay doi logic BillGo, khong thay doi database.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>feat(worker): add feature registry and dynamic module menu system</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -692,9 +720,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEC9037B-EFE6-49F5-A5F3-F97E00C66B25}">
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{CEC9037B-EFE6-49F5-A5F3-F97E00C66B25}">
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
@@ -704,7 +732,7 @@
     <col min="6" max="6" width="59" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" s="1" customFormat="1" ns3:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -724,7 +752,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ns3:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -738,7 +766,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ns3:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -758,7 +786,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ns3:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -776,6 +804,34 @@
       </c>
       <c r="F4" t="s">
         <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Worker Dynamic Menu</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Trang Tho sinh menu tu Feature Registry. BillGo chi hien khi tho co lich su/du lieu thu cuoc.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Giam hard-code menu, chuan bi mo rong module lau dai.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>feat(worker): add feature registry and dynamic module menu system</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -784,9 +840,9 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FE72BEA-FB82-4065-A82E-8E80ACFB3A0B}">
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{2FE72BEA-FB82-4065-A82E-8E80ACFB3A0B}">
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
@@ -796,7 +852,7 @@
     <col min="6" max="6" width="59" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" s="1" customFormat="1" ns3:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -816,7 +872,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ns3:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -830,7 +886,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ns3:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -850,7 +906,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ns3:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -868,6 +924,34 @@
       </c>
       <c r="F4" t="s">
         <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>BillGo menu visibility</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Khong doi nghiep vu thu cuoc. Chi thay dieu kien hien thi menu BillGo dua tren du lieu cua tho.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Tai khoan chua dung BillGo khong thay module khong lien quan.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>feat(worker): add feature registry and dynamic module menu system</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -876,9 +960,9 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73AD43CE-C0B8-4E8A-BE78-46E5E8BA5D1B}">
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{73AD43CE-C0B8-4E8A-BE78-46E5E8BA5D1B}">
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
@@ -888,7 +972,7 @@
     <col min="6" max="6" width="59" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" s="1" customFormat="1" ns3:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -908,7 +992,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ns3:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -925,7 +1009,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ns3:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -945,7 +1029,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ns3:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -963,6 +1047,34 @@
       </c>
       <c r="F4" t="s">
         <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Worker Feature Registry</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Khong tao migration. Layout doc du lieu hien co tu workers, billgo_subscriptions va billgo_receivables.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Tranh thay doi schema khi chua can.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>feat(worker): add feature registry and dynamic module menu system</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1009,9 +1121,9 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A759B5AA-E445-44B2-84E8-3B69A2E43B9A}">
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{A759B5AA-E445-44B2-84E8-3B69A2E43B9A}">
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
@@ -1021,7 +1133,7 @@
     <col min="6" max="6" width="59" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" s="1" customFormat="1" ns3:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1041,7 +1153,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ns3:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1058,7 +1170,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ns3:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1078,7 +1190,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ns3:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1096,6 +1208,34 @@
       </c>
       <c r="F4" t="s">
         <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Feature Registry cho module tho</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Moi module khai bao id, nhan, icon, quyen, dieu kien du lieu trong registry.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Module moi chi can dang ky cau hinh thay vi sua menu thu cong.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>feat(worker): add feature registry and dynamic module menu system</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(billgo): implement postpaid billing cycle with due date management
</commit_message>
<xml_diff>
--- a/ThoDenNgay_Product_Bible.xlsx
+++ b/ThoDenNgay_Product_Bible.xlsx
@@ -595,7 +595,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{2631304A-15A0-4692-B08D-1B98A6A6FAC0}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -714,6 +714,34 @@
         </is>
       </c>
     </row>
+    <row r="6" spans="1:6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Commit 2 BillGo postpaid</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Da them helper tinh ky, API tao BillGo, migration backfill va UI hien thi ky/han.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Khong thay doi menu Worker.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>feat(billgo): implement postpaid billing cycle with due date management</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -721,7 +749,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{CEC9037B-EFE6-49F5-A5F3-F97E00C66B25}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -834,6 +862,34 @@
         </is>
       </c>
     </row>
+    <row r="6" spans="1:6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>BillGo postpaid billing</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Moi ky thu cuoc hien thi ky su dung, han thanh toan, so tien va trang thai.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Thong nhat nghiep vu dung truoc - thu sau.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>feat(billgo): implement postpaid billing cycle with due date management</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -841,7 +897,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{2FE72BEA-FB82-4065-A82E-8E80ACFB3A0B}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -954,6 +1010,34 @@
         </is>
       </c>
     </row>
+    <row r="6" spans="1:6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Internet / BillGo</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Ky su dung ket thuc truoc, han thanh toan la ngay 20 thang ke tiep.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Phu hop mo hinh thu cuoc Internet tra sau.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>feat(billgo): implement postpaid billing cycle with due date management</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -961,7 +1045,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{73AD43CE-C0B8-4E8A-BE78-46E5E8BA5D1B}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1074,6 +1158,34 @@
       <c r="F5" t="inlineStr">
         <is>
           <t>feat(worker): add feature registry and dynamic module menu system</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>billgo_receivables</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Nang check status, backfill period_start/period_end/due_date; khong xoa du lieu cu.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Can chay migration_billgo_postpaid_cycles.sql tren Supabase.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>feat(billgo): implement postpaid billing cycle with due date management</t>
         </is>
       </c>
     </row>
@@ -1122,7 +1234,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{A759B5AA-E445-44B2-84E8-3B69A2E43B9A}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1235,6 +1347,34 @@
       <c r="F5" t="inlineStr">
         <is>
           <t>feat(worker): add feature registry and dynamic module menu system</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>BillGo dung truoc - thu sau</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Due date khong con la ngay bat dau ky ma la ngay 20 thang sau period_end.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Giam nham lan giua ky su dung va ngay thu tien.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>feat(billgo): implement postpaid billing cycle with due date management</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(worker): filter worker modules and services by approved categories
</commit_message>
<xml_diff>
--- a/ThoDenNgay_Product_Bible.xlsx
+++ b/ThoDenNgay_Product_Bible.xlsx
@@ -595,7 +595,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{2631304A-15A0-4692-B08D-1B98A6A6FAC0}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -742,6 +742,34 @@
         </is>
       </c>
     </row>
+    <row r="7" spans="1:6">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2">
+        <v>46213</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Fix worker category visibility</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Sua serviceMatchesSpecialties strict mode, registry requiresSpecialty va filter services trong worker dashboard.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Khong thay doi database.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>fix(worker): filter worker modules and services by approved categories</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -749,7 +777,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{CEC9037B-EFE6-49F5-A5F3-F97E00C66B25}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -890,6 +918,34 @@
         </is>
       </c>
     </row>
+    <row r="7" spans="1:6">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2">
+        <v>46213</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Worker category filtering</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Trang tho chi hien module/dich vu dung voi specialties cua tho.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Giam nham lan khi tho chi dang ky mot so nganh.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>fix(worker): filter worker modules and services by approved categories</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -897,7 +953,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{2FE72BEA-FB82-4065-A82E-8E80ACFB3A0B}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1035,6 +1091,34 @@
       <c r="F6" t="inlineStr">
         <is>
           <t>feat(billgo): implement postpaid billing cycle with due date management</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2">
+        <v>46213</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Tho / Dich vu</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Tao viec nhanh loc danh sach dich vu theo nganh nghe da duyet; thieu nganh thi fallback an toan.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Dam bao tho khong nhan/tao viec ngoai nganh.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>fix(worker): filter worker modules and services by approved categories</t>
         </is>
       </c>
     </row>
@@ -1234,7 +1318,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{A759B5AA-E445-44B2-84E8-3B69A2E43B9A}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1375,6 +1459,34 @@
       <c r="F6" t="inlineStr">
         <is>
           <t>feat(billgo): implement postpaid billing cycle with due date management</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2">
+        <v>46213</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Feature Registry specialties</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Dynamic Menu phai resolve theo specialties va data conditions, khong hien module chuyen biet khi chua co nganh.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Mo rong module sau nay co dieu kien ro rang.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>fix(worker): filter worker modules and services by approved categories</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(worker): prevent cross-category service matches
</commit_message>
<xml_diff>
--- a/ThoDenNgay_Product_Bible.xlsx
+++ b/ThoDenNgay_Product_Bible.xlsx
@@ -595,7 +595,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{2631304A-15A0-4692-B08D-1B98A6A6FAC0}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -770,6 +770,33 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr" s="2">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Fixed worker service/category filtering after dynamic menu rollout.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Workers should see only relevant services for their registered industries.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Affects worker menu and quick job/service selection.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -777,7 +804,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{CEC9037B-EFE6-49F5-A5F3-F97E00C66B25}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -946,6 +973,38 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr" s="2">
+        <is>
+          <t>Worker specialization filtering</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Worker UI only shows services matching registered/approved categories; generic child names no longer broaden matches.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>fix(worker): prevent cross-category service matches</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -953,7 +1012,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{2FE72BEA-FB82-4065-A82E-8E80ACFB3A0B}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1119,6 +1178,33 @@
       <c r="F7" t="inlineStr">
         <is>
           <t>fix(worker): filter worker modules and services by approved categories</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr" s="2">
+        <is>
+          <t>Tho</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Worker registered for Internet/Camera only sees Internet/Camera service choices and related worker modules.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>fix(worker): prevent cross-category service matches</t>
         </is>
       </c>
     </row>
@@ -1318,7 +1404,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{A759B5AA-E445-44B2-84E8-3B69A2E43B9A}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1490,15 +1576,42 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr" s="2">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Do not match worker services by generic child label across categories.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Avoid showing unrelated industries on worker PC/mobile screens.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>fix(worker): prevent cross-category service matches</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66436295-822F-41CE-8B74-4C18F3EB1C84}">
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{66436295-822F-41CE-8B74-4C18F3EB1C84}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5.140625" bestFit="1" customWidth="1"/>
@@ -1508,7 +1621,7 @@
     <col min="6" max="6" width="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" s="1" customFormat="1" ns3:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1526,6 +1639,28 @@
       </c>
       <c r="F1" s="1" t="s">
         <v>5</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr" s="1">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr" s="1">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr" s="1">
+        <is>
+          <t>Do not use generic service leaf names such as Lap dat or Sua chua as global worker-category matches.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr" s="1">
+        <is>
+          <t>They exist in multiple industries and cause unrelated services to appear.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(worker-sales): keep BillGo out of inventory sales
</commit_message>
<xml_diff>
--- a/ThoDenNgay_Product_Bible.xlsx
+++ b/ThoDenNgay_Product_Bible.xlsx
@@ -595,7 +595,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{2631304A-15A0-4692-B08D-1B98A6A6FAC0}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -797,6 +797,38 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Removed BillGo from worker inventory/sales flow</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Da go UI BillGo kho hang va ep p_create_billgo=false khi tao don ban.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Khong doi schema; chi thay doi nghiep vu va UI.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>fix(worker-sales): keep BillGo out of inventory sales</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -804,7 +836,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{CEC9037B-EFE6-49F5-A5F3-F97E00C66B25}">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1005,6 +1037,38 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Worker inventory/sales</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Kho hang va don ban cua tho khong con tuy chon tao BillGo.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>BillGo la module thu cuoc rieng, khong tron voi ban hang vat tu.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>fix(worker-sales): keep BillGo out of inventory sales</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1012,7 +1076,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{2FE72BEA-FB82-4065-A82E-8E80ACFB3A0B}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1205,6 +1269,38 @@
       <c r="E8" t="inlineStr">
         <is>
           <t>fix(worker): prevent cross-category service matches</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Tho / Kho hang / Ban hang</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>San pham kho va don ban chi phuc vu ban hang cua tho; khong danh dau thu dinh ky va khong tao lich BillGo.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Tranh tao cong no/thu cuoc sai ngu canh khi tho chi ban vat tu.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>fix(worker-sales): keep BillGo out of inventory sales</t>
         </is>
       </c>
     </row>
@@ -1404,7 +1500,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{A759B5AA-E445-44B2-84E8-3B69A2E43B9A}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1600,6 +1696,38 @@
       <c r="E8" t="inlineStr">
         <is>
           <t>fix(worker): prevent cross-category service matches</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>BillGo separate from worker sales inventory</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Khong cho bat BillGo trong form san pham kho hoac don ban cua tho.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>BillGo chi duoc quan ly trong module BillGo rieng.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>fix(worker-sales): keep BillGo out of inventory sales</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: tự động tạo mã sản phẩm theo danh mục
</commit_message>
<xml_diff>
--- a/ThoDenNgay_Product_Bible.xlsx
+++ b/ThoDenNgay_Product_Bible.xlsx
@@ -595,7 +595,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{2631304A-15A0-4692-B08D-1B98A6A6FAC0}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -829,6 +829,23 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>feat: tự động tạo mã sản phẩm theo danh mục</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Cập nhật UI form thêm/sửa sản phẩm, helper tạo mã, retry trùng mã, migration backfill dữ liệu cũ.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -836,7 +853,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{CEC9037B-EFE6-49F5-A5F3-F97E00C66B25}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1069,6 +1086,28 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Worker inventory</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Thêm sản phẩm tự sinh mã theo danh mục: NET, CAM, PC, PRI, SP; mã hiển thị sau khi chọn danh mục và có tùy chọn nhập mã riêng.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>feat: tự động tạo mã sản phẩm theo danh mục</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1076,7 +1115,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{2FE72BEA-FB82-4065-A82E-8E80ACFB3A0B}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1304,6 +1343,28 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Product code policy</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Mã sản phẩm duy nhất trong phạm vi worker_id + sku; mỗi thợ có thể dùng cùng mã với thợ khác; sửa sản phẩm không tự đổi mã.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>feat: tự động tạo mã sản phẩm theo danh mục</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1311,7 +1372,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{73AD43CE-C0B8-4E8A-BE78-46E5E8BA5D1B}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1452,6 +1513,28 @@
       <c r="F6" t="inlineStr">
         <is>
           <t>feat(billgo): implement postpaid billing cycle with due date management</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>worker_inventory_products</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Giữ ràng buộc UNIQUE(worker_id, sku); thêm migration backfill SKU rỗng theo danh mục và mã lớn nhất hiện có.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>supabase/migration_worker_inventory_product_codes.sql</t>
         </is>
       </c>
     </row>
@@ -1500,7 +1583,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{A759B5AA-E445-44B2-84E8-3B69A2E43B9A}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1728,6 +1811,28 @@
       <c r="F9" t="inlineStr">
         <is>
           <t>fix(worker-sales): keep BillGo out of inventory sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Worker product code</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Dùng trường sku hiện có làm mã sản phẩm để không ảnh hưởng tồn kho, đơn bán hàng và lịch sử giao dịch.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>feat: tự động tạo mã sản phẩm theo danh mục</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(worker-dashboard): add today stats
</commit_message>
<xml_diff>
--- a/ThoDenNgay_Product_Bible.xlsx
+++ b/ThoDenNgay_Product_Bible.xlsx
@@ -595,7 +595,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{2631304A-15A0-4692-B08D-1B98A6A6FAC0}">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -846,6 +846,23 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>feat(worker-dashboard): add today stats</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Cập nhật app/worker/page.tsx và tài liệu release cho thống kê hôm nay.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -853,7 +870,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{CEC9037B-EFE6-49F5-A5F3-F97E00C66B25}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1108,6 +1125,28 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Worker Dashboard</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Bảng điều khiển thợ hiển thêm thống kê hôm nay: khách hàng, đánh giá trung bình, tổng tiền đã thu.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>feat(worker-dashboard): add today stats</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1115,7 +1154,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{2FE72BEA-FB82-4065-A82E-8E80ACFB3A0B}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1362,6 +1401,28 @@
       <c r="D10" t="inlineStr">
         <is>
           <t>feat: tự động tạo mã sản phẩm theo danh mục</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Worker daily stats</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Tổng tiền hôm nay/tháng này ưu tiên payment paid_at; nếu chưa có payment thì fallback theo giá trị job hoàn thành.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>feat(worker-dashboard): add today stats</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1644,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{A759B5AA-E445-44B2-84E8-3B69A2E43B9A}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1833,6 +1894,28 @@
       <c r="D10" t="inlineStr">
         <is>
           <t>feat: tự động tạo mã sản phẩm theo danh mục</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Worker dashboard UI</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Giữ dashboard gọn, dùng nhãn ngắn và định dạng tiền compact k/tr cho mobile.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>feat(worker-dashboard): add today stats</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(worker-dashboard): optimize mobile stats layout
</commit_message>
<xml_diff>
--- a/ThoDenNgay_Product_Bible.xlsx
+++ b/ThoDenNgay_Product_Bible.xlsx
@@ -595,7 +595,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{2631304A-15A0-4692-B08D-1B98A6A6FAC0}">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -863,6 +863,23 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>feat(worker-dashboard): optimize mobile stats layout</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Cập nhật app/worker/page.tsx, CHANGELOG, RELEASE_NOTES và workbook cho layout mobile dashboard thợ.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -870,7 +887,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{CEC9037B-EFE6-49F5-A5F3-F97E00C66B25}">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1147,6 +1164,28 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Worker Dashboard</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Thống kê dashboard thợ hiển thị Tháng hiện tại ở trên và Hôm nay kèm ngày ở dưới trong cùng card.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>feat(worker-dashboard): optimize mobile stats layout</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1154,7 +1193,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{2FE72BEA-FB82-4065-A82E-8E80ACFB3A0B}">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1423,6 +1462,28 @@
       <c r="D11" t="inlineStr">
         <is>
           <t>feat(worker-dashboard): add today stats</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Worker mobile workflow</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Thợ có nút nổi Tạo việc trên mobile để mở nhanh form tạo việc cho khách quen.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>feat(worker-dashboard): optimize mobile stats layout</t>
         </is>
       </c>
     </row>
@@ -1644,7 +1705,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{A759B5AA-E445-44B2-84E8-3B69A2E43B9A}">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1916,6 +1977,28 @@
       <c r="D11" t="inlineStr">
         <is>
           <t>feat(worker-dashboard): add today stats</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Worker dashboard mobile density</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Ưu tiên giảm chiều cao dashboard trên mobile và giữ CTA tạo việc luôn dễ bấm.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>feat(worker-dashboard): optimize mobile stats layout</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(worker): show old backlog jobs
</commit_message>
<xml_diff>
--- a/ThoDenNgay_Product_Bible.xlsx
+++ b/ThoDenNgay_Product_Bible.xlsx
@@ -595,7 +595,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{2631304A-15A0-4692-B08D-1B98A6A6FAC0}">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -880,6 +880,23 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>feat(worker): show old backlog jobs</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Cập nhật app/worker/jobs/page.tsx, worker layout, dashboard quick job anchor và registry menu mobile.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -887,7 +904,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{CEC9037B-EFE6-49F5-A5F3-F97E00C66B25}">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1186,6 +1203,28 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Worker Tồn việc</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Trang thợ có nút Tồn việc trên mobile để mở danh sách việc cũ chưa làm; nút + mở khu vực tạo việc nhanh.</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>feat(worker): show old backlog jobs</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1193,7 +1232,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{2FE72BEA-FB82-4065-A82E-8E80ACFB3A0B}">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1487,6 +1526,28 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Worker backlog definition</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Tồn việc chỉ tính các job chưa hoàn thành có ngày tạo/lịch hẹn trước tháng hiện tại; việc trong tháng hiện tại không hiển thị ở mục này.</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>feat(worker): show old backlog jobs</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1494,7 +1555,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{73AD43CE-C0B8-4E8A-BE78-46E5E8BA5D1B}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1657,6 +1718,33 @@
       <c r="D7" t="inlineStr">
         <is>
           <t>supabase/migration_worker_inventory_product_codes.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>jobs</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Không đổi schema; danh sách Tồn việc dùng bảng jobs hiện có, lọc theo worker_id, trạng thái chưa hoàn thành và mốc trước đầu tháng hiện tại.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>No migration required</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>feat(worker): show old backlog jobs</t>
         </is>
       </c>
     </row>
@@ -1705,7 +1793,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{A759B5AA-E445-44B2-84E8-3B69A2E43B9A}">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1999,6 +2087,28 @@
       <c r="D12" t="inlineStr">
         <is>
           <t>feat(worker-dashboard): optimize mobile stats layout</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Worker mobile navigation</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Giữ 5 nút mobile; đổi Công việc thành Tồn việc để thể hiện các việc cũ chưa làm, còn nút + dành cho tạo việc nhanh.</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>feat(worker): show old backlog jobs</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(worker-inventory): filter category suggestions by specialty
</commit_message>
<xml_diff>
--- a/ThoDenNgay_Product_Bible.xlsx
+++ b/ThoDenNgay_Product_Bible.xlsx
@@ -595,7 +595,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{2631304A-15A0-4692-B08D-1B98A6A6FAC0}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -897,6 +897,23 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>feat(worker-inventory): filter category suggestions by specialty</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Cập nhật lib/worker-inventory.ts và form kho hàng để gợi ý danh mục theo workers.specialties.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -904,7 +921,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{CEC9037B-EFE6-49F5-A5F3-F97E00C66B25}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1225,6 +1242,28 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Worker Inventory</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Form thêm/sửa sản phẩm gợi ý danh mục theo chuyên môn của thợ, thay vì hiển thị toàn bộ danh mục.</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>feat(worker-inventory): filter category suggestions by specialty</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1232,7 +1271,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{2FE72BEA-FB82-4065-A82E-8E80ACFB3A0B}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1548,6 +1587,28 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Inventory category suggestions</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Danh mục kho chỉ là gợi ý nhập liệu; thợ vẫn có thể nhập danh mục riêng nếu cửa hàng cần.</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>feat(worker-inventory): filter category suggestions by specialty</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1555,7 +1616,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{73AD43CE-C0B8-4E8A-BE78-46E5E8BA5D1B}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1745,6 +1806,33 @@
       <c r="E8" t="inlineStr">
         <is>
           <t>feat(worker): show old backlog jobs</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>worker_inventory_products.category</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Không đổi schema; tiếp tục lưu category dạng text trên sản phẩm kho.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>No migration required</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>feat(worker-inventory): filter category suggestions by specialty</t>
         </is>
       </c>
     </row>
@@ -1793,7 +1881,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{A759B5AA-E445-44B2-84E8-3B69A2E43B9A}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -2109,6 +2197,28 @@
       <c r="D13" t="inlineStr">
         <is>
           <t>feat(worker): show old backlog jobs</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Inventory UX</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Không hiển danh sách danh mục tổng thể cho mọi thợ; ưu tiên danh sách ngắn theo chuyên môn để dễ chọn trên mobile.</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>feat(worker-inventory): filter category suggestions by specialty</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(worker-dashboard): shorten today stat label
</commit_message>
<xml_diff>
--- a/ThoDenNgay_Product_Bible.xlsx
+++ b/ThoDenNgay_Product_Bible.xlsx
@@ -595,7 +595,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{2631304A-15A0-4692-B08D-1B98A6A6FAC0}">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -914,6 +914,23 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>chore(worker-dashboard): shorten today stat label</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Cập nhật app/worker/page.tsx và tài liệu release cho nhãn thống kê Hôm nay.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -921,7 +938,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{CEC9037B-EFE6-49F5-A5F3-F97E00C66B25}">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1264,6 +1281,28 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Worker Dashboard</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Thống kê Hôm nay trên dashboard thợ chỉ hiển thị ngày, không hiển tháng.</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>chore(worker-dashboard): shorten today stat label</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1271,7 +1310,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{2FE72BEA-FB82-4065-A82E-8E80ACFB3A0B}">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1609,6 +1648,28 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Worker daily stats label</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Dữ liệu thống kê không đổi; chỉ rút gọn nhãn hiển thị Hôm nay theo số ngày.</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>chore(worker-dashboard): shorten today stat label</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1616,7 +1677,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{73AD43CE-C0B8-4E8A-BE78-46E5E8BA5D1B}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1833,6 +1894,33 @@
       <c r="E9" t="inlineStr">
         <is>
           <t>feat(worker-inventory): filter category suggestions by specialty</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>worker dashboard stats</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Không đổi schema hoặc truy vấn; chỉ đổi format nhãn ngày trên UI.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>No migration required</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>chore(worker-dashboard): shorten today stat label</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1969,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{A759B5AA-E445-44B2-84E8-3B69A2E43B9A}">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -2219,6 +2307,28 @@
       <c r="D14" t="inlineStr">
         <is>
           <t>feat(worker-inventory): filter category suggestions by specialty</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Worker Dashboard mobile UI</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Giữ nhãn Hôm nay ngắn hơn bằng cách chỉ hiển thị ngày, vì card đã có ngữ cảnh Tháng hiện tại.</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>chore(worker-dashboard): shorten today stat label</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(worker): add availability toggle
</commit_message>
<xml_diff>
--- a/ThoDenNgay_Product_Bible.xlsx
+++ b/ThoDenNgay_Product_Bible.xlsx
@@ -595,7 +595,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{2631304A-15A0-4692-B08D-1B98A6A6FAC0}">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -931,6 +931,23 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>feat(worker): add availability toggle</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Cập nhật dashboard thợ, header thợ, admin gán việc, types và migration_worker_availability.sql.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -938,7 +955,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{CEC9037B-EFE6-49F5-A5F3-F97E00C66B25}">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1303,6 +1320,28 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Worker Dashboard</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Bảng điều khiển thợ có nút Online/Offline; đèn sáng khi Online và tối khi Offline.</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>feat(worker): add availability toggle</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1310,7 +1349,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{2FE72BEA-FB82-4065-A82E-8E80ACFB3A0B}">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1670,6 +1709,28 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Worker availability</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Offline là tạm nghỉ nhận việc mới, không phải bị khóa tài khoản; thợ vẫn xem việc đang làm và tạo việc nhanh.</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>feat(worker): add availability toggle</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1677,7 +1738,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{73AD43CE-C0B8-4E8A-BE78-46E5E8BA5D1B}">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1921,6 +1982,33 @@
       <c r="E10" t="inlineStr">
         <is>
           <t>chore(worker-dashboard): shorten today stat label</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>workers.is_available</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Thêm cột is_available BOOLEAN NOT NULL DEFAULT TRUE, cập nhật policy việc pending và worker_accept_job để chặn thợ Offline nhận việc mới.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>supabase/migration_worker_availability.sql</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>feat(worker): add availability toggle</t>
         </is>
       </c>
     </row>
@@ -1969,7 +2057,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{A759B5AA-E445-44B2-84E8-3B69A2E43B9A}">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -2329,6 +2417,28 @@
       <c r="D15" t="inlineStr">
         <is>
           <t>chore(worker-dashboard): shorten today stat label</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Worker rest mode</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Dùng cờ is_available riêng thay vì đổi workers.status để không ảnh hưởng luồng duyệt pending/active/blocked.</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>feat(worker): add availability toggle</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(worker-inventory): allow category rename
</commit_message>
<xml_diff>
--- a/ThoDenNgay_Product_Bible.xlsx
+++ b/ThoDenNgay_Product_Bible.xlsx
@@ -595,7 +595,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{2631304A-15A0-4692-B08D-1B98A6A6FAC0}">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -948,6 +948,23 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>feat(worker-inventory): allow category rename</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Cập nhật app/worker/inventory/page.tsx và tài liệu release cho thao tác sửa danh mục kho.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -955,7 +972,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{CEC9037B-EFE6-49F5-A5F3-F97E00C66B25}">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1342,6 +1359,28 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Worker Inventory</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Thợ có thể sửa tên danh mục kho đang dùng nếu nhập nhầm.</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>feat(worker-inventory): allow category rename</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1349,7 +1388,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{2FE72BEA-FB82-4065-A82E-8E80ACFB3A0B}">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1731,6 +1770,28 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Inventory category correction</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Giữ danh mục kho là text linh hoạt; sửa tên danh mục sẽ cập nhật các sản phẩm của chính thợ đang dùng danh mục cũ.</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>feat(worker-inventory): allow category rename</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1738,7 +1799,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{73AD43CE-C0B8-4E8A-BE78-46E5E8BA5D1B}">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -2009,6 +2070,33 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>feat(worker): add availability toggle</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>worker_inventory_products.category</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Không đổi schema; thao tác sửa danh mục là UPDATE category theo worker_id và tên danh mục cũ.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>No migration required</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>feat(worker-inventory): allow category rename</t>
         </is>
       </c>
     </row>
@@ -2057,7 +2145,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{A759B5AA-E445-44B2-84E8-3B69A2E43B9A}">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -2439,6 +2527,28 @@
       <c r="D16" t="inlineStr">
         <is>
           <t>feat(worker): add availability toggle</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Inventory category UX</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Không tạo module CRUD danh mục riêng; chỉ thêm đổi tên danh mục đang dùng để sửa lỗi nhập.</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>feat(worker-inventory): allow category rename</t>
         </is>
       </c>
     </row>

</xml_diff>